<commit_message>
Test de Raiz unitaria. Todas deben aplicarse diferencias y logaritmos, se hizo mediante ADF y KPSS.
</commit_message>
<xml_diff>
--- a/outputs/resultados_raiz_unitaria.xlsx
+++ b/outputs/resultados_raiz_unitaria.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -456,10 +456,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C2" t="n">
-        <v>0.6915039640500688</v>
+        <v>0.7784379491522979</v>
       </c>
       <c r="D2" t="n">
         <v>0.01</v>
@@ -482,13 +482,13 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C3" t="n">
-        <v>0.7482543586416214</v>
+        <v>0.4206235033509499</v>
       </c>
       <c r="D3" t="n">
-        <v>0.01</v>
+        <v>0.01962927247032002</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -508,10 +508,10 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
+        <v>0.9989058849521039</v>
       </c>
       <c r="D4" t="n">
         <v>0.01</v>
@@ -534,10 +534,10 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C5" t="n">
-        <v>0.21536726896341</v>
+        <v>0.8249051176829643</v>
       </c>
       <c r="D5" t="n">
         <v>0.01</v>
@@ -560,10 +560,10 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C6" t="n">
-        <v>0.9502747020581239</v>
+        <v>0.2011420186227076</v>
       </c>
       <c r="D6" t="n">
         <v>0.01</v>
@@ -586,10 +586,10 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C7" t="n">
-        <v>0.9150616644041252</v>
+        <v>0.9853896259778411</v>
       </c>
       <c r="D7" t="n">
         <v>0.01</v>
@@ -612,10 +612,10 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>0.998652083050922</v>
       </c>
       <c r="D8" t="n">
         <v>0.01</v>
@@ -638,22 +638,22 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C9" t="n">
-        <v>0.02053281218998596</v>
+        <v>0.07673215927099805</v>
       </c>
       <c r="D9" t="n">
-        <v>0.1</v>
+        <v>0.0163707823703453</v>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Usar esta serie</t>
+          <t>Revisar transformación</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C10" t="n">
         <v>1</v>
@@ -690,10 +690,10 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C11" t="n">
-        <v>0.1895571658231284</v>
+        <v>0.4544790657957452</v>
       </c>
       <c r="D11" t="n">
         <v>0.01</v>
@@ -716,22 +716,22 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C12" t="n">
-        <v>0.01565180921956285</v>
+        <v>0.0829657170314842</v>
       </c>
       <c r="D12" t="n">
         <v>0.1</v>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Mixta</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Usar esta serie</t>
+          <t>Revisar transformación</t>
         </is>
       </c>
     </row>
@@ -742,10 +742,10 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="C13" t="n">
-        <v>0.7999409873350116</v>
+        <v>0.9744582541484981</v>
       </c>
       <c r="D13" t="n">
         <v>0.01</v>
@@ -758,6 +758,270 @@
       <c r="F13" t="inlineStr">
         <is>
           <t>Revisar transformación</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>D_ln_Vol_comerciales</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" t="inlineStr"/>
+      <c r="D14" t="inlineStr"/>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>D_Mora_comerciales</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>D_ln_Vol_consumo</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" t="inlineStr"/>
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>D_Mora_consumo</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" t="inlineStr"/>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>D_ln_Vol_hipotecarios</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" t="inlineStr"/>
+      <c r="D18" t="inlineStr"/>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>D_Mora_hipotecarios</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" t="inlineStr"/>
+      <c r="D19" t="inlineStr"/>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>D_ln_Vol_microcreditos</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>0</v>
+      </c>
+      <c r="C20" t="inlineStr"/>
+      <c r="D20" t="inlineStr"/>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>D_Mora_microcreditos</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>D_ln_Vol_total</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>D_Mora_total</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>D_Tasa_Ref</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr"/>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>D_ln_PBI_Desestacionalizado</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>0</v>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr"/>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>No evaluada</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>No existe en el archivo</t>
         </is>
       </c>
     </row>
@@ -849,19 +1113,19 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>-1.157744317184888</v>
+        <v>-0.9285123777731472</v>
       </c>
       <c r="D2" t="n">
-        <v>0.6915039640500688</v>
+        <v>0.7784379491522979</v>
       </c>
       <c r="E2" t="n">
         <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>245</v>
+        <v>211</v>
       </c>
       <c r="G2" t="n">
-        <v>2363.041468144287</v>
+        <v>2031.471701027056</v>
       </c>
       <c r="H2" t="b">
         <v>0</v>
@@ -872,13 +1136,13 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>-3.457326071908813</v>
+        <v>-3.46172743446274</v>
       </c>
       <c r="K2" t="n">
-        <v>-2.873410402808354</v>
+        <v>-2.875337467779996</v>
       </c>
       <c r="L2" t="n">
-        <v>-2.573095980841316</v>
+        <v>-2.574124089081557</v>
       </c>
     </row>
     <row r="3">
@@ -893,16 +1157,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>2.121931551436471</v>
+        <v>1.929659087934888</v>
       </c>
       <c r="D3" t="n">
         <v>0.01</v>
       </c>
       <c r="E3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="b">
@@ -935,19 +1199,19 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>-1.013647073554258</v>
+        <v>-1.720419746649569</v>
       </c>
       <c r="D4" t="n">
-        <v>0.7482543586416214</v>
+        <v>0.4206235033509499</v>
       </c>
       <c r="E4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="G4" t="n">
-        <v>-1844.761456990575</v>
+        <v>-1597.187989675328</v>
       </c>
       <c r="H4" t="b">
         <v>0</v>
@@ -958,13 +1222,13 @@
         </is>
       </c>
       <c r="J4" t="n">
-        <v>-3.458366327573048</v>
+        <v>-3.462657673481232</v>
       </c>
       <c r="K4" t="n">
-        <v>-2.873866099917713</v>
+        <v>-2.875744421584133</v>
       </c>
       <c r="L4" t="n">
-        <v>-2.573339078569377</v>
+        <v>-2.574341231409875</v>
       </c>
     </row>
     <row r="5">
@@ -979,16 +1243,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1.293386487980579</v>
+        <v>0.6330780028264797</v>
       </c>
       <c r="D5" t="n">
-        <v>0.01</v>
+        <v>0.01962927247032002</v>
       </c>
       <c r="E5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F5" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="b">
@@ -1021,19 +1285,19 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>3.597925273778108</v>
+        <v>2.229462821146138</v>
       </c>
       <c r="D6" t="n">
-        <v>1</v>
+        <v>0.9989058849521039</v>
       </c>
       <c r="E6" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F6" t="n">
-        <v>243</v>
+        <v>203</v>
       </c>
       <c r="G6" t="n">
-        <v>2004.113377398812</v>
+        <v>1491.101435179605</v>
       </c>
       <c r="H6" t="b">
         <v>0</v>
@@ -1044,13 +1308,13 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>-3.457550507794775</v>
+        <v>-3.462980134086401</v>
       </c>
       <c r="K6" t="n">
-        <v>-2.873508732301353</v>
+        <v>-2.875885461947131</v>
       </c>
       <c r="L6" t="n">
-        <v>-2.573148434859185</v>
+        <v>-2.574416489844451</v>
       </c>
     </row>
     <row r="7">
@@ -1065,16 +1329,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>2.239141630408995</v>
+        <v>2.147951329685946</v>
       </c>
       <c r="D7" t="n">
         <v>0.01</v>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F7" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="b">
@@ -1107,19 +1371,19 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>-2.175205230520301</v>
+        <v>-0.7800743775246606</v>
       </c>
       <c r="D8" t="n">
-        <v>0.21536726896341</v>
+        <v>0.8249051176829643</v>
       </c>
       <c r="E8" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F8" t="n">
-        <v>236</v>
+        <v>203</v>
       </c>
       <c r="G8" t="n">
-        <v>-2554.304511764716</v>
+        <v>-2242.189430483471</v>
       </c>
       <c r="H8" t="b">
         <v>0</v>
@@ -1130,13 +1394,13 @@
         </is>
       </c>
       <c r="J8" t="n">
-        <v>-3.458366327573048</v>
+        <v>-3.462980134086401</v>
       </c>
       <c r="K8" t="n">
-        <v>-2.873866099917713</v>
+        <v>-2.875885461947131</v>
       </c>
       <c r="L8" t="n">
-        <v>-2.573339078569377</v>
+        <v>-2.574416489844451</v>
       </c>
     </row>
     <row r="9">
@@ -1151,16 +1415,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>1.660509974219366</v>
+        <v>1.8015866047429</v>
       </c>
       <c r="D9" t="n">
         <v>0.01</v>
       </c>
       <c r="E9" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F9" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="b">
@@ -1193,19 +1457,19 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>-0.09153987572324152</v>
+        <v>-2.214172242180671</v>
       </c>
       <c r="D10" t="n">
-        <v>0.9502747020581239</v>
+        <v>0.2011420186227076</v>
       </c>
       <c r="E10" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>236</v>
+        <v>205</v>
       </c>
       <c r="G10" t="n">
-        <v>1819.82732864336</v>
+        <v>1186.506894280747</v>
       </c>
       <c r="H10" t="b">
         <v>0</v>
@@ -1216,13 +1480,13 @@
         </is>
       </c>
       <c r="J10" t="n">
-        <v>-3.458366327573048</v>
+        <v>-3.462657673481232</v>
       </c>
       <c r="K10" t="n">
-        <v>-2.873866099917713</v>
+        <v>-2.875744421584133</v>
       </c>
       <c r="L10" t="n">
-        <v>-2.573339078569377</v>
+        <v>-2.574341231409875</v>
       </c>
     </row>
     <row r="11">
@@ -1237,16 +1501,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>2.316303409491713</v>
+        <v>2.127708870920662</v>
       </c>
       <c r="D11" t="n">
         <v>0.01</v>
       </c>
       <c r="E11" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F11" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="b">
@@ -1279,19 +1543,19 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>-0.3695398043019344</v>
+        <v>0.5173029936844897</v>
       </c>
       <c r="D12" t="n">
-        <v>0.9150616644041252</v>
+        <v>0.9853896259778411</v>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="F12" t="n">
-        <v>242</v>
+        <v>212</v>
       </c>
       <c r="G12" t="n">
-        <v>-2302.250224698942</v>
+        <v>-2073.942160985713</v>
       </c>
       <c r="H12" t="b">
         <v>0</v>
@@ -1302,13 +1566,13 @@
         </is>
       </c>
       <c r="J12" t="n">
-        <v>-3.457664132155201</v>
+        <v>-3.461577578407847</v>
       </c>
       <c r="K12" t="n">
-        <v>-2.873558510596022</v>
+        <v>-2.875271898983725</v>
       </c>
       <c r="L12" t="n">
-        <v>-2.573174989413292</v>
+        <v>-2.574089103773585</v>
       </c>
     </row>
     <row r="13">
@@ -1323,16 +1587,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>1.972083491238565</v>
+        <v>1.656586951759731</v>
       </c>
       <c r="D13" t="n">
         <v>0.01</v>
       </c>
       <c r="E13" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F13" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="b">
@@ -1365,19 +1629,19 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>2.837644259917045</v>
+        <v>1.984212900450403</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0.998652083050922</v>
       </c>
       <c r="E14" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F14" t="n">
-        <v>237</v>
+        <v>202</v>
       </c>
       <c r="G14" t="n">
-        <v>2704.410860072144</v>
+        <v>2136.730528106838</v>
       </c>
       <c r="H14" t="b">
         <v>0</v>
@@ -1388,13 +1652,13 @@
         </is>
       </c>
       <c r="J14" t="n">
-        <v>-3.458246798239911</v>
+        <v>-3.463143790625264</v>
       </c>
       <c r="K14" t="n">
-        <v>-2.873813746108132</v>
+        <v>-2.875957037982105</v>
       </c>
       <c r="L14" t="n">
-        <v>-2.573311149032385</v>
+        <v>-2.574454682874228</v>
       </c>
     </row>
     <row r="15">
@@ -1409,16 +1673,16 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>2.259345216778854</v>
+        <v>2.222305426278492</v>
       </c>
       <c r="D15" t="n">
         <v>0.01</v>
       </c>
       <c r="E15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F15" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="b">
@@ -1451,36 +1715,36 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>-3.190641580132758</v>
+        <v>-2.684651144042706</v>
       </c>
       <c r="D16" t="n">
-        <v>0.02053281218998596</v>
+        <v>0.07673215927099805</v>
       </c>
       <c r="E16" t="n">
         <v>6</v>
       </c>
       <c r="F16" t="n">
-        <v>245</v>
+        <v>211</v>
       </c>
       <c r="G16" t="n">
-        <v>-2273.542674312095</v>
+        <v>-1985.041795169672</v>
       </c>
       <c r="H16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>Estacionaria</t>
+          <t>No estacionaria</t>
         </is>
       </c>
       <c r="J16" t="n">
-        <v>-3.457326071908813</v>
+        <v>-3.46172743446274</v>
       </c>
       <c r="K16" t="n">
-        <v>-2.873410402808354</v>
+        <v>-2.875337467779996</v>
       </c>
       <c r="L16" t="n">
-        <v>-2.573095980841316</v>
+        <v>-2.574124089081557</v>
       </c>
     </row>
     <row r="17">
@@ -1495,24 +1759,24 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.2409506048076376</v>
+        <v>0.6689213939262016</v>
       </c>
       <c r="D17" t="n">
-        <v>0.1</v>
+        <v>0.0163707823703453</v>
       </c>
       <c r="E17" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F17" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>Estacionaria</t>
+          <t>No estacionaria</t>
         </is>
       </c>
       <c r="J17" t="n">
@@ -1537,19 +1801,19 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4.126479462172904</v>
+        <v>2.786782361185446</v>
       </c>
       <c r="D18" t="n">
         <v>1</v>
       </c>
       <c r="E18" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F18" t="n">
-        <v>238</v>
+        <v>203</v>
       </c>
       <c r="G18" t="n">
-        <v>2809.068435346571</v>
+        <v>2144.208388859876</v>
       </c>
       <c r="H18" t="b">
         <v>0</v>
@@ -1560,13 +1824,13 @@
         </is>
       </c>
       <c r="J18" t="n">
-        <v>-3.458128284586202</v>
+        <v>-3.462980134086401</v>
       </c>
       <c r="K18" t="n">
-        <v>-2.873761835239286</v>
+        <v>-2.875885461947131</v>
       </c>
       <c r="L18" t="n">
-        <v>-2.573283455970623</v>
+        <v>-2.574416489844451</v>
       </c>
     </row>
     <row r="19">
@@ -1581,16 +1845,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2.298075704305082</v>
+        <v>2.212088272074322</v>
       </c>
       <c r="D19" t="n">
         <v>0.01</v>
       </c>
       <c r="E19" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F19" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="b">
@@ -1623,19 +1887,19 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>-2.247215461536245</v>
+        <v>-1.654913690995402</v>
       </c>
       <c r="D20" t="n">
-        <v>0.1895571658231284</v>
+        <v>0.4544790657957452</v>
       </c>
       <c r="E20" t="n">
         <v>8</v>
       </c>
       <c r="F20" t="n">
-        <v>243</v>
+        <v>209</v>
       </c>
       <c r="G20" t="n">
-        <v>-2395.440141629344</v>
+        <v>-2078.173632390064</v>
       </c>
       <c r="H20" t="b">
         <v>0</v>
@@ -1646,13 +1910,13 @@
         </is>
       </c>
       <c r="J20" t="n">
-        <v>-3.457550507794775</v>
+        <v>-3.462031503678967</v>
       </c>
       <c r="K20" t="n">
-        <v>-2.873508732301353</v>
+        <v>-2.875470502482713</v>
       </c>
       <c r="L20" t="n">
-        <v>-2.573148434859185</v>
+        <v>-2.574195072686065</v>
       </c>
     </row>
     <row r="21">
@@ -1667,16 +1931,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1.141119053083222</v>
+        <v>1.347320313843621</v>
       </c>
       <c r="D21" t="n">
         <v>0.01</v>
       </c>
       <c r="E21" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F21" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G21" t="inlineStr"/>
       <c r="H21" t="b">
@@ -1709,36 +1973,36 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>-3.283082991366597</v>
+        <v>-2.650694461659326</v>
       </c>
       <c r="D22" t="n">
-        <v>0.01565180921956285</v>
+        <v>0.0829657170314842</v>
       </c>
       <c r="E22" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="F22" t="n">
-        <v>247</v>
+        <v>205</v>
       </c>
       <c r="G22" t="n">
-        <v>-179.3889340732254</v>
+        <v>-216.7672266116225</v>
       </c>
       <c r="H22" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Estacionaria</t>
+          <t>No estacionaria</t>
         </is>
       </c>
       <c r="J22" t="n">
-        <v>-3.457105309726321</v>
+        <v>-3.462657673481232</v>
       </c>
       <c r="K22" t="n">
-        <v>-2.873313676101283</v>
+        <v>-2.875744421584133</v>
       </c>
       <c r="L22" t="n">
-        <v>-2.573044382468161</v>
+        <v>-2.574341231409875</v>
       </c>
     </row>
     <row r="23">
@@ -1753,16 +2017,16 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.2599296906456028</v>
+        <v>0.1343722035399938</v>
       </c>
       <c r="D23" t="n">
         <v>0.1</v>
       </c>
       <c r="E23" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F23" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G23" t="inlineStr"/>
       <c r="H23" t="b">
@@ -1795,19 +2059,19 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>-0.8629108364945092</v>
+        <v>0.2407795419182538</v>
       </c>
       <c r="D24" t="n">
-        <v>0.7999409873350116</v>
+        <v>0.9744582541484981</v>
       </c>
       <c r="E24" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F24" t="n">
-        <v>243</v>
+        <v>213</v>
       </c>
       <c r="G24" t="n">
-        <v>1231.539352945095</v>
+        <v>678.2421169752158</v>
       </c>
       <c r="H24" t="b">
         <v>0</v>
@@ -1818,13 +2082,13 @@
         </is>
       </c>
       <c r="J24" t="n">
-        <v>-3.457550507794775</v>
+        <v>-3.461429147102264</v>
       </c>
       <c r="K24" t="n">
-        <v>-2.873508732301353</v>
+        <v>-2.875206950587861</v>
       </c>
       <c r="L24" t="n">
-        <v>-2.573148434859185</v>
+        <v>-2.5740544497344</v>
       </c>
     </row>
     <row r="25">
@@ -1839,16 +2103,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>2.348308678079867</v>
+        <v>2.285471498847192</v>
       </c>
       <c r="D25" t="n">
         <v>0.01</v>
       </c>
       <c r="E25" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F25" t="n">
-        <v>252</v>
+        <v>218</v>
       </c>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="b">

</xml_diff>